<commit_message>
feat: Add ISIN support for companies and market sweeps
- Introduced ISIN (International Securities Identification Number) field in the Company and MarketSweepCompany models.
- Updated the company detail and settings templates to display and edit ISIN.
- Implemented ISIN validation and normalization utilities.
- Enhanced the market sweep upload functionality to include ISIN handling, ensuring proper validation during file imports.
- Added admin functionality to set ISINs for sweep rows via API.
- Updated frontend components to display ISIN alongside company tickers and allow ISIN input for admins.
- Included new styles for ISIN display in the investment journey and market sweep interfaces.
</commit_message>
<xml_diff>
--- a/data/market-sweeps/Brazil.xlsx
+++ b/data/market-sweeps/Brazil.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +117,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:F213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -518,6 +519,11 @@
           <t>exchange</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>isin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -545,6 +551,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -572,6 +579,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -599,6 +607,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -626,6 +635,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -653,6 +663,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -680,6 +691,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -707,6 +719,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -734,6 +747,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -761,6 +775,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -788,6 +803,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -815,6 +831,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -842,6 +859,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -869,6 +887,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -896,6 +915,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -923,6 +943,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -950,6 +971,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -977,6 +999,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1004,6 +1027,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1031,6 +1055,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1058,6 +1083,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1085,6 +1111,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1112,6 +1139,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1139,6 +1167,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1166,6 +1195,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1193,6 +1223,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1220,6 +1251,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1247,6 +1279,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1274,6 +1307,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1301,6 +1335,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1328,6 +1363,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1355,6 +1391,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1382,6 +1419,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1409,6 +1447,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1436,6 +1475,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1463,6 +1503,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1490,6 +1531,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1517,6 +1559,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1544,6 +1587,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1571,6 +1615,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1598,6 +1643,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1625,6 +1671,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1652,6 +1699,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1679,6 +1727,7 @@
           <t>B3 - BDR</t>
         </is>
       </c>
+      <c r="F44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1706,6 +1755,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1733,6 +1783,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -1760,6 +1811,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1787,6 +1839,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1814,6 +1867,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1841,6 +1895,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1868,6 +1923,7 @@
           <t>B3 - BDR</t>
         </is>
       </c>
+      <c r="F51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1895,6 +1951,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -1922,6 +1979,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1949,6 +2007,7 @@
           <t>B3 - BDR</t>
         </is>
       </c>
+      <c r="F54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -1976,6 +2035,7 @@
           <t>B3 - BDR</t>
         </is>
       </c>
+      <c r="F55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2003,6 +2063,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2030,6 +2091,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2057,6 +2119,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2084,6 +2147,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2111,6 +2175,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2138,6 +2203,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2165,6 +2231,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2192,6 +2259,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2219,6 +2287,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2246,6 +2315,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2273,6 +2343,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2300,6 +2371,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2327,6 +2399,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2354,6 +2427,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2381,6 +2455,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2408,6 +2483,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2435,6 +2511,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -2462,6 +2539,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2489,6 +2567,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2516,6 +2595,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2543,6 +2623,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2570,6 +2651,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2597,6 +2679,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -2624,6 +2707,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2651,6 +2735,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -2678,6 +2763,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2705,6 +2791,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -2732,6 +2819,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2759,6 +2847,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -2786,6 +2875,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2813,6 +2903,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -2840,6 +2931,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2867,6 +2959,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -2894,6 +2987,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2921,6 +3015,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -2948,6 +3043,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2975,6 +3071,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -3002,6 +3099,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3029,6 +3127,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -3056,6 +3155,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3083,6 +3183,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -3110,6 +3211,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3137,6 +3239,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -3164,6 +3267,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3191,6 +3295,7 @@
           <t>B3 - Traditional</t>
         </is>
       </c>
+      <c r="F100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -3218,6 +3323,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3245,6 +3351,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -3272,6 +3379,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3299,6 +3407,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -3326,6 +3435,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3353,6 +3463,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -3380,6 +3491,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3407,6 +3519,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3434,6 +3547,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3461,6 +3575,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -3488,6 +3603,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3515,6 +3631,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -3542,6 +3659,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -3569,6 +3687,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -3596,6 +3715,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -3623,6 +3743,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -3650,6 +3771,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -3677,6 +3799,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -3704,6 +3827,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3731,6 +3855,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -3758,6 +3883,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -3785,6 +3911,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -3812,6 +3939,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -3839,6 +3967,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -3866,6 +3995,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3893,6 +4023,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -3920,6 +4051,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -3947,6 +4079,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -3974,6 +4107,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -4001,6 +4135,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -4028,6 +4163,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -4055,6 +4191,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -4082,6 +4219,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4109,6 +4247,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -4136,6 +4275,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -4163,6 +4303,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -4190,6 +4331,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4217,6 +4359,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -4244,6 +4387,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -4271,6 +4415,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -4298,6 +4443,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4325,6 +4471,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -4352,6 +4499,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -4379,6 +4527,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -4406,6 +4555,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -4433,6 +4583,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -4460,6 +4611,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -4487,6 +4639,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -4514,6 +4667,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -4541,6 +4695,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -4568,6 +4723,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -4595,6 +4751,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -4622,6 +4779,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -4649,6 +4807,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -4676,6 +4835,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -4703,6 +4863,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -4730,6 +4891,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -4757,6 +4919,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -4784,6 +4947,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -4811,6 +4975,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -4838,6 +5003,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -4865,6 +5031,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -4892,6 +5059,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -4919,6 +5087,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -4946,6 +5115,7 @@
           <t>B3 - Level 2</t>
         </is>
       </c>
+      <c r="F165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -4973,6 +5143,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -5000,6 +5171,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -5027,6 +5199,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -5054,6 +5227,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -5081,6 +5255,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -5108,6 +5283,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -5135,6 +5311,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -5162,6 +5339,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -5189,6 +5367,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -5216,6 +5395,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -5243,6 +5423,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -5270,6 +5451,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -5297,6 +5479,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -5324,6 +5507,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -5351,6 +5535,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -5378,6 +5563,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -5405,6 +5591,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -5432,6 +5619,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -5459,6 +5647,7 @@
           <t>B3</t>
         </is>
       </c>
+      <c r="F184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -5486,6 +5675,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -5513,6 +5703,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -5540,6 +5731,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -5567,6 +5759,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -5594,6 +5787,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -5621,6 +5815,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -5648,6 +5843,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -5675,6 +5871,7 @@
           <t>B3 - Level 1</t>
         </is>
       </c>
+      <c r="F192" s="7" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -5702,6 +5899,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F193" s="7" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -5729,6 +5927,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F194" s="7" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -5756,6 +5955,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F195" s="7" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -5783,6 +5983,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F196" s="7" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -5810,6 +6011,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F197" s="7" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -5837,6 +6039,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F198" s="7" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -5864,6 +6067,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F199" s="7" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -5891,6 +6095,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F200" s="7" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -5918,6 +6123,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F201" s="7" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -5945,6 +6151,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F202" s="7" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -5972,6 +6179,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F203" s="7" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -5999,6 +6207,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F204" s="7" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -6026,6 +6235,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F205" s="7" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -6053,6 +6263,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F206" s="7" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -6080,6 +6291,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F207" s="7" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -6107,6 +6319,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F208" s="7" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -6134,6 +6347,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F209" s="7" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -6161,6 +6375,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F210" s="7" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -6188,6 +6403,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F211" s="7" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -6215,6 +6431,7 @@
           <t>B3 - Novo Mercado</t>
         </is>
       </c>
+      <c r="F212" s="7" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -6242,6 +6459,7 @@
           <t>B3 - BDR</t>
         </is>
       </c>
+      <c r="F213" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E213"/>

</xml_diff>